<commit_message>
Revisiones y correcciones de keywords. 12/02/2026 09:53 am
</commit_message>
<xml_diff>
--- a/Output/reporte_REAL.xlsx
+++ b/Output/reporte_REAL.xlsx
@@ -437,7 +437,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3">
@@ -448,7 +448,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>-0.13</t>
+          <t>-0.08</t>
         </is>
       </c>
     </row>
@@ -460,7 +460,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-02-11T10:46:53.058492</t>
+          <t>2026-02-12T09:51:45.540427</t>
         </is>
       </c>
     </row>
@@ -497,7 +497,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-1.9125</v>
+        <v>-1.165494736842105</v>
       </c>
     </row>
     <row r="3">
@@ -507,7 +507,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-2.86875</v>
+        <v>-1.74899298245614</v>
       </c>
     </row>
     <row r="4">
@@ -517,7 +517,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.9562499999999999</v>
+        <v>0.5585298245614037</v>
       </c>
     </row>
     <row r="5">
@@ -527,7 +527,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.9562499999999999</v>
+        <v>-0.6666140350877193</v>
       </c>
     </row>
     <row r="6">
@@ -537,7 +537,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-2.295</v>
+        <v>-1.394442105263158</v>
       </c>
     </row>
   </sheetData>
@@ -551,7 +551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -609,26 +609,26 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-02-10T17:00:00</t>
+          <t>2026-02-12T15:11:01</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Kristi Noem Firma Contrato Para la Compra de Acero para el Muro entre EUA y México - N+</t>
+          <t>México pide a EU revisar aranceles a acero, aluminio y sector automotriz: Ebrard - Tiempo La Noticia</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>N+</t>
+          <t>Tiempo La Noticia Digital</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxPamxsVURNOGU0aGN5Z1g2QVpTeFZxcFNFY2tJS01MWC05ZWF5bG1tU1hnN0RRSG9Fd2VxM2hqVDBNd1pwdThmeUJkUXVCM19DdEVhSHFiaENnLUdkVXhyYTd6WS1pdy1sM09jUXhoU3BJTVBCUVdTNWIzWTZyb1R1ZWdPLXduNFVmdDhhbURERl9YUkVCR28yamVVZmFrWEpHdGNNeWZYM3RLSmR3SjY5VGJjTWhJWUpVcU4tZW9JS1dkbFMxQkgyMGlCb0F3WUZvdUh6amd3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxNajFrU3ZnYTV0NE4yd1ZBLWNidEExT2JicmdjVWhWaWJRU1Q5TWUzT3MxVW5rWjE3bFo0YjVUTy1UUDdtN3NtbHdxSng5RHNTMy1uSTZPSklxeHRMNzhxQ2NkUWNQWFpnVWg5OEQ0TktlbDBSNTJpb2JIczEwSjUtRXhBUm1lTkJWVXVtbWNaSDlfQzJkbWlraVFsQ3dUWE5IVk9IU0xfRVhKZjVjalV3dg?oc=5</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>-0.34</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -636,37 +636,37 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>-0</v>
+        <v>-3.4</v>
       </c>
       <c r="H2" t="n">
-        <v>-0</v>
+        <v>-5.100000000000001</v>
       </c>
       <c r="I2" t="n">
-        <v>-0</v>
+        <v>1.7</v>
       </c>
       <c r="J2" t="n">
-        <v>-0</v>
+        <v>-1.7</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-02-08T21:20:47</t>
+          <t>2026-02-12T14:07:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Jóvenes escalan chimenea de AHMSA en Monclova y se viralizan en redes - vanguardia.com.mx</t>
+          <t>Ternium toma el control de Usiminas tras comprar la participación de Nippon en Brasil - La Nación</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>vanguardia.com.mx</t>
+          <t>La Nación</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxOeHNyWFhVTVVoNGcySjIzSTZXSGsxM2pfc2VCMC1rbDgweU9odG9IaGp3Y1ROU1lWTGZQbHRyQXVWVWRwX1o1aXduamZ3QzJUOEpGZlVqZEFqU0t3XzBITmU2bmNyX3dMVW5pUWlkaE9hUy05SkU1YS1WX215RWZZMS1BMkt3ZVRQSG5CaUJXckx2QV9lZWJyeXdKbGlxUER6T25zVDBHU3loTEFkdnBKSThpSU5ka2duTllFSXVfSFFYUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi3AFBVV95cUxOd2s0M1NwcVpIQVdGNDhEdXQ2RzR4Wkc0VHFkcTZCZmxoNl84NkVqYWpXdURHOWlObmRuLWxnRWljU3BzdmtXX3dqS283dDJqQ3JMeU1nU2ROOXpERTFoWHgzQ09aM0hyRkV5NjJYU1ZybHNmbkRya1ZoX0V2czk4YXUta3FkSzlURjA1blpvME16N1JVclY4V0d2d3RsMVRVSWcteE5fLVp3OWpsM29Ra2xndnA3emFpeGI5TnoxTDczZ0psYlpBaWxSQUdzVHc5Q1I0YVF2RjRCWDVS?oc=5</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -693,22 +693,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-02-08T14:00:00</t>
+          <t>2026-02-12T13:56:03</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Entre fuego y acero, la herencia artesanal de los cuchilleros de Sayula de México - UDG TV</t>
+          <t>Ternium toma el control de una acerera de Brasil - Ejes</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>UDG TV</t>
+          <t>Ejes</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPQWVLdjlMX1J0MHY5dHNrMjA3WlJTTWJkV1o4N010UGR5d3dtUzVpc3RUenYwR1BoeG9vNllDLXN5dU1sb2hsZjNFSkNtSE14aVJ3S2N0cXRxM1Q5d3M0ZERHay1KZFpVNm5mUDlGOWl2Y3VoNC11anZSRUd5T2p5QW1IZVBJS1RWVFR3dUsyNzRnYXo0dks3bHp3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxQVUxyZk9HTE4wQXhYeEV6dUpoamlSM3FpWkFMNVB6VHNINW9KbTFiOVNMejZtLUVnX2duek04MllENHpYUmRYWEp3R245Qk5kYjdZTGRYUWNnMWpabmJtR3NBUFJtaWM0MDFBLUxNeW1XcDhwd2hLVzRiT1VMamgyeW1hWk5FVUhyR1RranNadzNGQlpJR3BqWS1WMzM?oc=5</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -735,43 +735,2269 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-02-05T10:28:49</t>
+          <t>2026-02-12T12:15:18</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Estados Unidos ultima un acuerdo con México para permitir un cupo de acero sin aranceles del 50% - M</t>
+          <t>China y México mantienen conversaciones en medio de tensiones comerciales por aranceles - El Economi</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>El Economista</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxOT0lpWWt2MXo2Ym1fbHdrVEF6V2loR25WSkZkLXVuTHNtOUp5dW41bWZ0a2V3dFAyY25ONmhGMHlrT1JMRE1fWmNIS0hRSXAwM1dUa3UwblBNR0dySkktRmpKdF9aTVFoZXpVbFF4MlEtRmwzSTd2Yzc1OWxUNXBYUFJ6empNLTY3NlFKZFVmcXhwX2ptWUdZZmZIOTNPbm02a2RENmpUb0h3LTFIbEtBeERzWGFxZlBPLVdsOUQyaXlIZ1Utekl5UUFsWndXdHJwUGlJ0gHYAUFVX3lxTE1aZVMxYU9VdjdqUzMzUW9aVEdMVWN4elpjX013R1RkQ0VDb2V3WjRyMEx4VFhYRjRDUTlVb29XVFBxNkxtRGZJZ0hpV2V5LXVuOGRadE5NSHRPRGdkRzJaVUN2bjNkUEpnbHdVUnVXN3FfQlhtZGhheDFUTHdNdE81aXdNZEozYTdKampaajJNZWdtc1RnTUx0Tmw5UWY4ME5iRHROLXJhLTZoSVFiUUl1TzdZTDd4T3E2WHZLSjNKWkZkdG5NcGdmWmpGNkxhR2RtQndUck1iVg?oc=5</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>-0.34</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>-3.4</v>
+      </c>
+      <c r="H5" t="n">
+        <v>-5.100000000000001</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="J5" t="n">
+        <v>-1.7</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-02-12T11:16:54</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>CEO de Thyssenkrupp: Aranceles mejoran panorama del acero y negociaciones con Jindal - Investing.com</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Investing.com México - Finanzas, Bolsa y Forex</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi3AFBVV95cUxQNXhjRHJNNzRkSHN2eTNWcGdaX1FCYzRLNGtvQkx2Si1fcjB3X2sxS1dYWnhpUWtZdnU4SmlwR01ZVklSUGdQOHg3Y0RzanFSUWgza25VSmNwaERiOWdJbk11c0NjMnJ2X2NiaFJwam9KVEoyTHNTNTl2Y1lvZFhHZkhQMmJiLUdJcWc4RDAxamVmcmJWSHBVN3F1MlBnS0hWYWJ3TlpwTFRTcWRwYXoyZExGVjZITjhsTnVxeEh1YVF3TnlJd0l0WWFsT1ZGZkdQTXhoZzB6MnRobnNO?oc=5</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>0.6599999999999999</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>positivo</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>-6.6</v>
+      </c>
+      <c r="H6" t="n">
+        <v>-9.899999999999999</v>
+      </c>
+      <c r="I6" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="J6" t="n">
+        <v>-3.3</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-02-12T11:15:00</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Director ejecutivo de Thyssenkrupp: Aranceles impulsan la confianza en el acero y negociaciones con </t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Investing.com Español</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi-gFBVV95cUxONkdtb3FEbmNsUmZWVEdHdFBJazNWQ0R1bTFzek9uOVJBSkR3cVFRTTRJTFA2VERoYV9KYXBuWm9hdWdHc2RpV3E0U0ZfdWswYzMxelBlVjlwUUFZdGszTFNocGY5c1hlcDY4ZnR2Q284cnM1WjBGaG40WldhcmZTYmJ0MjNyVFVzRzhJZzNuaWVDYzkwVHhQeDk2Zk9pbHVaVlNQLW5TcHF0cGxfTGg3WDlaS1dPZ1NUa0lBV0dTV1ZybEhaMUwtcC1rbDM2X0lWOEkwTGxSTXVvbmxtQkktMnZVLWZfa3Z0a1BLUWdaM3l1X25GNU9Ua2hR?oc=5</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>0.6599999999999999</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>positivo</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>-6.6</v>
+      </c>
+      <c r="H7" t="n">
+        <v>-9.899999999999999</v>
+      </c>
+      <c r="I7" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="J7" t="n">
+        <v>-3.3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-02-12T03:55:00</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Arcelormittal fuerza la subida de sus precios objetivo a lomos del escudo arancelario - TradingView</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>TradingView</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiaEFVX3lxTE96QmZVdjBPNDY1RXBtUUwxVDNKaktlODdpcXhhS043UHJZcFdIZDY4M1JmSHZuczR1ZFBSOUF0Q3R2MGprLVpkU3FJdDVRUGxrRFFFN0FwaDFuUnhpRU5IbnhlR09KWHNI?oc=5</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>-0.34</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>-3.4</v>
+      </c>
+      <c r="H8" t="n">
+        <v>-5.100000000000001</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="J8" t="n">
+        <v>-1.7</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-02-12T00:30:00</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Hay una grave persecución sindical y laboral en Coahuila: Mejía Berdeja - Sociedad Noticias</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Sociedad Noticias</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNRllJNURiZ0ZraXU5Ny0xc05WX3NJLUowT1U0NlQ3MERpeF9JU1gxZ21FTktVMEV3MGlKdmdvYndtdG9zZDdKRndJUi1fckFNRUx5aHJPOFQ5R0hFM0lKZ1RtLWJnZE0xc2tVb3FaYkwxaGMyZGZ5WW9VVm9RMjlta3UyLUh4R1RBdl85dlJFb2JyRmVaVDEydHpCZXBtR3JNQlNsYUlvVkhoUDdfamRLUmVn?oc=5</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-02-12T00:20:12</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Exige PT se Liquiden a extrabajadores de Altos Hornos de México Tras la Quiebra de la Empresa - Tecn</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Tecnoempresa</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxNUHJkdFFiaDBiLVlPOV9CczZlLWFIWFFVbGJOd2UycWNqeU5wdVNtazNGMTJDbVZPdm1qQmt5VlFUYXV6S2ItZ0tSYnZNNE1pOEhKa2pvWXFKaG5tb2ZWaFBjTWZfUlpVZm9mNFZPZGJ6Y0tFRVY2NklSTlRJWkV6UkF4cVBaR0prRXNIQTNfSzVsUW9RbHRGMjNOYmZudEMxUnVqQ0dDTGtQenpxRWlENHFqcjFidWc1ZEE?oc=5</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>negativo</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>-3</v>
+      </c>
+      <c r="H10" t="n">
+        <v>-4</v>
+      </c>
+      <c r="I10" t="n">
+        <v>-2</v>
+      </c>
+      <c r="J10" t="n">
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-02-11T23:16:00</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Inversionistas buscan adquirir AHMSA en Monclova: subasta el 27 de febrero - Periódico La Voz</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Periódico La Voz</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxNOUxFNHBERUNtdTdISXpQaE1wd1pQT2dpdk50cnBMN25fSnlvSDh6S012SVpNbEhqTzRDR0VOd3FvVG5OWEVONUJUZnUyaFh5aTE2VWU0REV0XzR1VDVIUjBzeW9qN0N2SEItRmEyS3M2LUt0eUtFT2wySGtSRGZrV2FHTlBicDc3Q2YwcE9nZWh3VERZZzNzOU52RmVFb1l4RHhfWlZ30gGrAUFVX3lxTE9YTFZZcGFEUHZsbXIxaHpPci1KTzJDbUU1NUwxc0VMR1p5aV9rdHFFRU5rcXVmU3B5MnhwVkFlbkFuWERTbUVBeUs0azN3Z1l3Qi0xX3RnTnIwWV9TcTJZWVFDWDFzMkJXNWp3VWRwbjdNNThBdmpGSERIUm55c0xlTFd4LXBkZzhGdGFlRklyRnFKOE1lOUhWczJWRjE0azloX2MtakVhNDM0WQ?oc=5</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J11" t="n">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-02-11T21:04:44</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Después de la polémica con la Casa Rosada, Techint concretó una fuerte inversión en Brasil - El Canc</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>El Canciller</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxPQjVYZ0ZLZ0JkbWVmXzQ1OF8wREpoZ1loWGhYY0hnejdhZ0tmUVE0RFA3SDBrd0ZzMG5GbTJya2JDcmFTN3BZQlJMQ0k4MnltZkx1dnMwaE9aclBGUkNhYmZOOTRkQlF2QkFqaVB1Zk91Vy1veVhtb2tlNDdzVXB4UHN1UTl6VFNpZXduM0JCMXpJY0JRUXdGa3k0REk1R1ExNURLcUJ3eGlXOHBobk1TS3VjY1Z0UXljQ0k4SHlia091VWxydk5VU0Z6WGVEdkViWTZBLThkSGwyd0JEMzRuVk4wa9IB8gFBVV95cUxPSHJGQ0pYbjdJN01oNThSRTlzT2tTSXZrTl9RSXZlUUFuUmZBdHRsSmRaWE1TZm5hZlBaVWNsVDY2VXBKZ3RkR1J2SDRMaFhuRkM0T0lDaUwtejM4bXkwNXpwZGlyS05pcjZfNmlqTUo3SW9WMXhfTmZPLXRxQ0xFUzBJS2I0SmFoLW1jSzRlMjhSQzZuME5WejJxcXlIRXhWRld6b2VUZ2NkRVZOWkdqMVVBSlZoaVdGY0ZNWVNNcjdJOV9PSjJLdlRMME56TS1TZVcwSXVONU5YTVdfS2Fnbk0tZnhVRC12LU04NHRIUnpvQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J12" t="n">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-02-11T20:35:00</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Avanza venta de AHMSA; compiten seis compradores por la siderúrgica - PostaMx</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>PostaMx</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPWHNSM1dUWHNGbkdVTlcwMHdlRVk1bzZWZGZiaVkyOTdpRDNqWHdmb1ljNk1sNjNWVGp0akJLTVRRY3ptZElHcGl5MktlODNCcG5saXhyd2RfZHZ0RzlzNV9MSlR0VlFzSjlNLVh6QTN5Zk5EdG9lNXEzbG93dG1RN295UVFSQVI5TmZaRVdfbWh3WEhRV0hMSGtzbHpyczBlMWVEUzA1THJycXlfX2RZ0gG0AUFVX3lxTE93eXF1V0ZvbWVhRndVaWtqVmtNVkJJbFZhcmhZZUZ6T3NoaGZ1aWhCSzZHX0NGWUFCLTVrWkFEbC12ZnBGb2s0a0x0SU81d0tsUmVITVd1OWNaT0RYZWpiak1pRkYxWG1UTGJpUHZXZ0ZPVWt5U3E1WnZvRmhNcnJNRXVoOFc5b2E4QTBINGc3TzNjX2dvbXU2aFdDajFIb3hIbkdBRjg3VlEzUHJlVzQzeThzZw?oc=5</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I13" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J13" t="n">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-02-11T18:54:23</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Rocca deja atrás la polémica con Milei: invierte US$ 315 millones en un gigante de Brasil y crece en</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Clarin.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxQZ0R1ZHJoQUN3dC1pMEhDZEYyLWdtcnFUMGd5ZkRQRmRMUEhNVkhJMmNDTnJMYWNIbmNaVktnVl9DOHptQ01mQVgzb3lBY3cwRDlJUE9BV0RRXzctd1NTWGR6T0JGcEMxTENfdVlMMnE3QlFBSW1SM2xnU3VEem5nM0ZwbDdwN3J1UXVqUXNKaFJxYS1FQUg1Y0NqTTZHMmVxc3JyYTIweUt4cWxidmhlakZoYVVWTlpTckdJLXczTVdReUp4OEIyay05VXk2UXEt?oc=5</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>positivo</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>3</v>
+      </c>
+      <c r="H14" t="n">
+        <v>4</v>
+      </c>
+      <c r="I14" t="n">
+        <v>2</v>
+      </c>
+      <c r="J14" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-02-11T18:34:00</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Confía Grupo de Defensa Laboral en venta de AHMSA durante subasta - INFO7</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>INFO7</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxOeDdxV2k1Yy1oa0xqRkRZRjdqYzYzdUlfejVKYVlZdWl3NVRCNVczeFdHYWVRWkdsMUJmUWVidEJleEVNMzhHT1dEMWpiUDFZaGlVcnJIMVZmM0wxeTBzUHFaYjJrVjBtVXl5OG1xd0hqWUtnaWZsZVVxVGJIempXeU42UHZZZ2pYYzlOWlFvQldCRnBWX01NWEhMeU5ndGswaWt0TE9qQmFib1E?oc=5</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J15" t="n">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-02-11T16:55:34</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Ampliación de convenios entre México y Brasil elevará más de 10% inversiones en ambos en sectores es</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>diariodetabasco.mx</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi8wFBVV95cUxNTXpOU2RGZkxHdTNTVkF2VWlzVGVzdEdBdDhzLVNEdmxwanJaTVB5UXd1elNRY0hSdkxubS14RWZCOGNwaVhYdTM3Y1pVR0ZVZXphY25SSV83RU1BZFJvS3NxcmJfUGp5U2NYMm00QXlZT3hlTUlBU0NuVnk1U18wd0Ruc21XSWxGVGxQeElWWHJPc3dWNU92ZVVpVHBSU3FYNFZzbzd2RkZpV1MxUGNTRE9xRDdFT0RrV2t0d1ZDTmRyOV9abFlVWUQ3OE9seERwSlRqWUxJVThTbjNERUVONFN3d01XYVRYVDRBZ0JBMFVTbmM?oc=5</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J16" t="n">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-02-11T15:31:31</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Ternium avanza en Brasil y adquiere las acciones de Usiminas - LM Neuquén</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>LM Neuquén</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxQYnhsb0s2NkI5SGdJWlB0YlhKOFZKME9rdVMyb1luUXVNSTU5S2lwTzhkLXA1UTBpME5pYzE2aHZpNWtJZVVOWUl6U21OQnNCVFZKVkZKbGNpS1hMMVJ3OFNqamN5SzdURjRDd0tLbE11SkhpWTJpbU95ay1fbl9nTHdsTDRlcWYyZ2tmbFFNalROeEFYMWVxUUZ4REN4NktI?oc=5</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J17" t="n">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-02-11T15:27:32</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Tras el cruce con el Gobierno, Techint se quedó con más del 70% de una de las principales siderúrgic</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Infobae</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi3gFBVV95cUxQeE1CTFdCc0s5c0trM05EVFYzSGl0aE5sZDlwcG5lZzY0bE4teXRCYkREamQxdl9McHd5eGNIeEZ3VmV4NTJtZjhfblRGaC1ncGFFcFhmWnVtSF91Q2RJZVpqS3I3ajIxUE5OLTdJbm52QTR0N1NBLVNYTHBkWFA4UXZvaDczN0pROHFqS0tMUGs0MjVQQk52THgtWDhGd1lHNGZwcXBMaU9OM2p5TDl5TXJmdDFWWXhOS29wTzNVVFI1U0JZRXloM0hzSVdBMl9DQ0ZOX3JsSTM2ZGdKMlHSAfgBQVVfeXFMUGloMVU0Um9kdVlJa2dQWnphRjZOMUpWVGF6ejgxWk9rNDA2Zm00UV8xbWJ4bWdQc1pEdlV3a3pXNnJDMjNGOGh5djZ0ejRQb2JObm1FMEd5d3hrRHlUWWdsNXNwTko4MEh4ZWZCRTcydExVUVhNZ0pGOFV5V1FkVUNwdXl3eDhpa1ZyYlNvMER2X2NFR0JXXy1sOWpVbGNjczRzaG1qbXFPT21pSnhqV2lMR29kVWR5OTctVkxOdWs4MEpWc1hxZG1jZk5CMFAxdkxtSlBORXl1RTY1X09yRG81dlFtX2k2OV9EY2NwbDdtd1RqS0hnTjQ?oc=5</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H18" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I18" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J18" t="n">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-02-11T12:00:01</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Trump amaga con aranceles de 100 % a farmacéuticas mexicanas; quiere su producción en EU - La Crónic</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>La Crónica de Hoy</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxPeDdqQWY5ckJuWkpYSXlxMkstNHRtRkFwUDZMcXZrVmZoMk92RHhEM29UeG5Zb1ZKUkFVMHVxVy1OYU11S0lMaUYwVzdGcHZEV01iNVlwNUFtbzBxaWVyUDZuOWRQY0xYbVc4bVhoTDRBS1UySXk4c3l3YmRnbUg3clVZZEJoM2Y3a0hfRkl2M1Fva2diR2dVTlhpZ05tMlVrRE9oS3ZwTmdPRmthRk5RUHl6aE9mRC1jVkh2ckdHd3lFeS13aW5keVd4bzg5QQ?oc=5</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>-0.51</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>-7.649999999999999</v>
+      </c>
+      <c r="H19" t="n">
+        <v>-11.475</v>
+      </c>
+      <c r="I19" t="n">
+        <v>3.825</v>
+      </c>
+      <c r="J19" t="n">
+        <v>-3.825</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-02-11T10:06:18</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Sugieren que personalidades de la vida pública en México sí tengan protección vehicular de alto nive</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Hoja de Ruta Digital</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxNNEVBUkRmR1FiaGpReF96cEVSM1lUTVBrd0dEWWdKRDYyVHJLU1FQTU50X2cyRFVUX2lhSWJndkd4R0xOOWVxMXJwM2VCVzFBQ3RMQXRKdWFPV3dCYk9ibndURFBMUlNMSVEweHJYRmZPRFpSZnJhSkZ0ak4za2RoN3hPeE9xZDI2b3U5ZkFEWnQ1OXFvVE1iTDdnY0pCT05ENFd2STdWU29lYy1EZnpBS0VrX0dtQjBJQ2lGUFJ5YVJ2VWxpU1pNbmNJWQ?oc=5</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H20" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I20" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J20" t="n">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-02-11T00:20:42</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>La Décima Sexta Zona Naval recibe visita de alumnos de la Escuela Primara “Voluntad de Acero” - Gent</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Gente del Balsas</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxPLWUtZjlMbV9KOUw5VEVJSUpiVnpsMVV5eVFDeGFqT0g0S09ZUmppRXZRMVdtTmk5bTFGSzJ0OV9wb0k0OTBQdlhhc19vWlhGLVlTQlVDXzVhcThGbmJBZGRzREhaV1g4QW1SdHY2bDZibl9iSTNZNllpdW1wRU5Lb1ZQOVF6YWdpN2N4ZlRfa3dQMDVxLVdxYVVFZ0RyVUJkcGxKbnAxdldxN0tqSDNjLW9xUDJhMUdkQXIzZThNZDEyVDFLYkhxNg?oc=5</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H21" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I21" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J21" t="n">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-02-11T00:00:00</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Futuro del T-MEC, en riesgo: Trump evalúa sacar a EU del tratado con México y Canadá</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>El Financiero</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://www.elfinanciero.com.mx/economia/2026/02/11/futuro-del-t-mec-en-riesgo-trump-evalua-sacar-a-eu-del-tratado-con-mexico-y-canada/</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>negativo</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>-3</v>
+      </c>
+      <c r="H22" t="n">
+        <v>-4</v>
+      </c>
+      <c r="I22" t="n">
+        <v>-2</v>
+      </c>
+      <c r="J22" t="n">
+        <v>-2</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-02-11T00:00:00</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Ampliación de convenios entre México y Brasil elevará más de 10% inversiones en ambos en sectores es</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Milenio</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://www.milenio.com/negocios/convenios-mexico-brasil-elevaran-inversiones-nuevo-ace</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>positivo</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>3</v>
+      </c>
+      <c r="H23" t="n">
+        <v>4</v>
+      </c>
+      <c r="I23" t="n">
+        <v>2</v>
+      </c>
+      <c r="J23" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-02-10T23:21:44</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Mientras se disipa la polémica por los caños, Techint se expande en la industria siderúrgica regiona</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>El Cronista</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxPVmV2dGVvaklKdHAyUkd6dFBlQjVoU0dkUmpXbkVXQ1RJeXEwOFU4RFVoNGlOcUtRaUpFZTA1cGFzQ25hS1UzZFpJUWdZckMyR1Z2ZEFuOTJVaFc4V3JSaUZMMjBoQXc4bm8tY2JMdWxPVGFrRmg2WURhU3NHd0l6Q0VENVlhS1Zrd1pIWUQzMm5kQTNOYU1UN3JGNGJYZ3NLb2EtYktSUjBGTktVSXAzbjFjME5tb2sybVNzUkk3V0pLR2VYNldyQnN0WEI0ZExI0gHrAUFVX3lxTE43MVNvdWxNTDNnV3AybWdoSlo0b0NGQXlsSTlReFZsWjlqVFVhYkRORTVPNWk2NzQxUlJ2eldxdnNUcFNPVm5TancyUU03RllHbkd3MThtV1I3UmprX3NJNko0S2dpTnpMNVowNHphQnR3S2hqYmMzSm9MNXY2N2w5S3lsdGlkNmE3T28zZ2txeENxYndIRlJ5RXlMdGY1LUxpcWI3bVo3WmhoT256alNXS3JfbHNvaWNGc0tJYkx5NlRkUHNsZDJXSHV5ZWRaZ1NRZkkzODcyUnpzTEN5YVUzNGw0bDNjdjRYd3c?oc=5</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H24" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I24" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J24" t="n">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-02-10T23:21:44</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Mientras se disipa la polémica por los caños, Techint se expande en la industria siderúrgica regiona</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>El Cronista</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxONzFTb3VsTUwzZ1dwMm1naEpaNG9DRkF5bEk5UXhWbFo5alRVYWJETkU1TzVpNjc0MVJSdnpXcXZzVHBTT1ZuU2p3MlFNN0ZZR25HdzE4bVdSN1Jqa19zSTZKNEtnaU56TDVaMDR6YUJ0d0toamJjM0pvTDV2NjdsOUt5bHRpZDZhN09vM2drcXhDcWJ3SEZSeUV5THRmNS1MaXFiN21aN1poaE9uempTV0tyX2xzb2ljRnNLSWJMeTZUZFBzbGQyV0h1eWVkWmdTUWZJMzg3MlJ6c0xDeWFVMzRsNGwzY3Y0WHd30gHrAUFVX3lxTE43MVNvdWxNTDNnV3AybWdoSlo0b0NGQXlsSTlReFZsWjlqVFVhYkRORTVPNWk2NzQxUlJ2eldxdnNUcFNPVm5TancyUU03RllHbkd3MThtV1I3UmprX3NJNko0S2dpTnpMNVowNHphQnR3S2hqYmMzSm9MNXY2N2w5S3lsdGlkNmE3T28zZ2txeENxYndIRlJ5RXlMdGY1LUxpcWI3bVo3WmhoT256alNXS3JfbHNvaWNGc0tJYkx5NlRkUHNsZDJXSHV5ZWRaZ1NRZkkzODcyUnpzTEN5YVUzNGw0bDNjdjRYd3c?oc=5</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H25" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I25" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J25" t="n">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-02-10T21:21:00</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Ternium completa adquisición de acciones de Usiminas por 315,2 millones de dólares - Investing.com E</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Investing.com Español</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxNd1VjUE5fbndlOGdvU2RyNXlpUGhrZ2czSnItbVVPUHVTZjl3bi1felNFWHEydmNqbFZRTUtXenk4UDdpbE5GS2FtekNJLXdwVFhCMkFUSEcwMmN3aHN4ZWVRb0hrZTNBdWVsd0dWZGxQX0IxMW9USmoxNFdIem10eDVBZkEwV0M4ZlhGT3JVa1VyNzZNZ3F4bWtlUlpMeVhHcDVpMGhmeXZxNHR3VVFtWGk4TVVMa0VpcGFsMHBKMWpDRFlQOGdiLVZtdUdncmpCWE1F?oc=5</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H26" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I26" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J26" t="n">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-02-10T17:00:00</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Kristi Noem Firma Contrato Para la Compra de Acero para el Muro entre EUA y México - N+</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>N+</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxPamxsVURNOGU0aGN5Z1g2QVpTeFZxcFNFY2tJS01MWC05ZWF5bG1tU1hnN0RRSG9Fd2VxM2hqVDBNd1pwdThmeUJkUXVCM19DdEVhSHFiaENnLUdkVXhyYTd6WS1pdy1sM09jUXhoU3BJTVBCUVdTNWIzWTZyb1R1ZWdPLXduNFVmdDhhbURERl9YUkVCR28yamVVZmFrWEpHdGNNeWZYM3RLSmR3SjY5VGJjTWhJWUpVcU4tZW9JS1dkbFMxQkgyMGlCb0F3WUZvdUh6amd3?oc=5</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H27" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I27" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J27" t="n">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-02-10T00:00:00</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Cárteles y barras bravas, los principales retos para autoridades mexicanas en la Copa del Mundo 2026</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Milenio</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>https://www.milenio.com/policia/retos-seguridad-copa-del-mundo-2026-mexico-cuales-son</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H28" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I28" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J28" t="n">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-02-10T00:00:00</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Carney contradice a Trump y afirma que ‘Canadá pagó por el puente’ que conecta con EU</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Forbes.com.mx</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>https://forbes.com.mx/carney-contradice-a-trump-y-afirma-que-canada-pago-por-el-puente-que-conecta-con-eu/</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="H29" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="J29" t="n">
+        <v>1.04</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-02-10T00:00:00</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>El Volkswagen Virtus 2026 ya tiene precio en México: el sucesor del Vento ofrece dos motores, tres v</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Motorpasión México</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>https://www.motorpasion.com.mx/industria/volkswagen-virtus-2026-precio-mexico</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G30" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H30" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I30" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J30" t="n">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-02-09T23:23:05</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Empleo formal en México registra en enero su peor inicio de año desde 2009 - bloomberglinea.com</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>bloomberglinea.com</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxNOFcyUXlOZTRTOXBHX0tMRnJtbHNLQXlZSVcwakZSUGdBQmFkTHFZRGxBUXljc1dxYjBpZldMbEEweGRBbXNDM09kSEtjQXNjT2tiUWtjZ2FuMEZlaklBMWx3aU5MTW0zQWRyVUxJTm54R1hvTXM0aFVEVWt3S0d1cjFlNTVHaU9FTUpUTnJ1aHZ4MjB5anhoVzFGU0VldTBreldHZWdaU0ZkVmdPWmpIdTJLNWpMSXhzczJBSi1ENmlJRjlqZUHSAdoBQVVfeXFMTTlTU2xaWENoZnh2NTVhbTNqb3RHbXJkcmMtWFhhSlZYYnhsWlRfdVZlb3k4c3JkTmpEeW1QVzUwSk03RDl1VXBNcTBhZ0pyME10clpPTDlsRUVkRjBWYlBuRHdaQ3lHbXJWRURjTVU5SjdWb0xackxpZ3pYYjkxaHBFR3N0X3Yya2xLeHY3eGF5R3pURnU2MVJQRjFoQldQWEpOc29RUUZVRC1PTGVYZV9FMVZlejVKbzlGS3ZraTJwNkJSR0dEU01IQlRfVTJOaW1iQVJZUTVITUE?oc=5</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H31" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I31" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J31" t="n">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-02-09T21:50:37</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Princess House busca emprendedores en Culiacán y promueve cocina saludable con acero inoxidable - de</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>debate.com.mx</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi7gFBVV95cUxQSjhxemJYWjhyTndoMlRzTmRjWnlNb2lWOGktbjhuaTRPQmJqTUtwdFZmSjVCZEhtQm42X2VKekZiVG16bXBqNkg1bUVsdXY5TWlCMjlhSDlKLVlQTFZ5ZVBROEsyRVRObWJwZnNxLUxfUzZhSlI5M0FxbGMxb3V5ZldvSGtESHh2SjVIZDRzbnh5dWdRcW9lMTRMSEt4YXBJQ3UzM2tsWGI5TTJRU2ZKODRvMGN6Y0xxNWtHb0RvLWhybXBCMGQ0U2xsSlZpNFFtWEh6TTBuOGtTemlkWG9UYkNKbndDZ0lzQ1JGYXpB0gHzAUFVX3lxTE91cWZDd2ZTWkxNZGV6VFgxOEhkYnBONExjaDJYWXI1ZW9QOFc2Rk5QSzlMSXUySERrbVZ6ckJpNjM3UjlLVVVSUG5MaFRyV1BHY0x4bkJIc2VZYllNNjE3Qm1TU1RiRnI1MlhDOFFaaWM3QkM5RmtOdktjejFsaEtFY01ZMmxGd2R2ZG1vS0M3OWx1bmhfSnQ5amhSREtOb21XQW04T2stV0RVS3FqM2stMmlDSTl4MGNqc2EtXzhzS3NydVlBcHFxbHZyN202dHp5N2hNZzBiN3djYUV3UTI3bDN3UkFiRzllSU40SE9xbmhxdw?oc=5</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H32" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I32" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J32" t="n">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-02-09T09:59:16</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Tubos Reunidos registra unas pérdidas de 71,3 millones de euros por los aranceles estadounidenses al</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
           <t>MSN</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiogNBVV95cUxPaExJTk5rcW1hc2R6emFudkwwMXBudWxGdHhONkJORUczQ0xwb05kQTdDUnZzS2xBZVVQY2RoQ0JvVHk2Z1NDTThiLVM3RWJJSXNmNm5ITmdCZnhkWHpaZlA5NTkzd0FVcG1IcUZtNDZBTnpKczlScjVhdHVGRmdCdklOOGRUakllWDgzZGhLM0o4aVp1eUZLdVlIazlnZEJrY0k1djU1a0FLbjlJcXI1NnZUd25VMGtWY25XdGdKNjJJU2hfNUJwNXBJZlVhQmVyVFN3NWdqS05TX2EwamJrMmFCZEdqNS1nTTc1WTR4RFlHSFVPOXY4cW1PNDhxVnZtb0d5REpyUzZseGNLalZkbzV4MjJ1ZXo5QzZ3Qk8xdEJfNjBDT0w1eFFkd3lyYjVoajJZWFJ4TlpBWDctTVkxYnpUTVJMZFFxaTl4aTFtbF8tdjJ1dmRkQUt2NTNnQjBDM1pKZGlqemdGejk2VHlVdWVFU2dQUVBKcE5Cc29WVVduZmZBVmJXc3E5YXFCdDdTSzQ2eHVnQVhfa21UbGdMeWtB?oc=5</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>-0.51</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>neutral</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
-        <v>-7.649999999999999</v>
-      </c>
-      <c r="H5" t="n">
-        <v>-11.475</v>
-      </c>
-      <c r="I5" t="n">
-        <v>3.825</v>
-      </c>
-      <c r="J5" t="n">
-        <v>-3.825</v>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi-AFBVV95cUxQWGd2c3B3X3ZadU9tMnp3cWFWSmMySUdMT3ZKTUIxQXRnMmpfWFZfZ3MySlZaNUJJZHhhck01TFVQX3ZMelhNc1ZNQUFsYXVaODVkM0U5aUpzU0V1S01lcFgySDhzNkotUl83OFZVd2ZMd1dRcm9fclZXYVF0VVh0eUdkQ3hmQVhlaXkyQ25fNkxzRFB5d2tvWC13MEZhLVhYZjFjNlZZR3dhZmhQY1YyelQ0Q3JVRmxUUFpsRTRJR3RyS0pURXlaYUREM0ctajFwSkZxUHFITEY1VEwtbEJUbmxxNjVHM0pzNG5iQ1ctYW9RWkFRb29adg?oc=5</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>negativo</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>-10</v>
+      </c>
+      <c r="H33" t="n">
+        <v>-15</v>
+      </c>
+      <c r="I33" t="n">
+        <v>5</v>
+      </c>
+      <c r="J33" t="n">
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-02-08T21:20:47</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Jóvenes escalan chimenea de AHMSA en Monclova y se viralizan en redes - vanguardia.com.mx</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>vanguardia.com.mx</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxOeHNyWFhVTVVoNGcySjIzSTZXSGsxM2pfc2VCMC1rbDgweU9odG9IaGp3Y1ROU1lWTGZQbHRyQXVWVWRwX1o1aXduamZ3QzJUOEpGZlVqZEFqU0t3XzBITmU2bmNyX3dMVW5pUWlkaE9hUy05SkU1YS1WX215RWZZMS1BMkt3ZVRQSG5CaUJXckx2QV9lZWJyeXdKbGlxUER6T25zVDBHU3loTEFkdnBKSThpSU5ka2duTllFSXVfSFFYUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H34" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I34" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J34" t="n">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-02-08T18:01:27</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>"Ilegales e injustificados", los aranceles de Trump a acero y aluminio: Canadá; hay "discusiones int</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>MSN</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilwNBVV95cUxQREFualdmQ1E5VHIyemE0V3VOdkxXd0xrVXpZcXhhVkpkM2RZVmhDaGJFNTBoZFNuX0FGbEpneHlta3p2S1BHTGN1dWFtVUxGUW9peU8wbVZyY1AwV055SGhxTGdEbTB2TFMwaHEwOTdsd2s1MlZfS2g5UVJoUUpEU2tkY3ZBQmY5ZU1hcWNxYjNQUHByOTJNVV9sSTc3dEVnSlZxZDdYd2lZTkhUMGRLSHdCVFlILVgwWHBCMWlfdF9fRUpPV3lsTFRyNEFqbVgyNXh6X0VsaU40VGZTZ2tQdVc4RjZrcERfVER1eUJJUzNwc0prU2hQcG96X1hyLXdRNEc0ZGpGZFpDbmdYcUswdEUzdFJOcFZ1ZnIwVG83c2pFS2E0bjVhTEw1ZG04UGdmRUg2a3ZJMnZzSU4xa3FOYjFqTk9JVGdBSzBGdkF1dHZDd2hYMjJld0RFQ3ZoNkFvSWhQOTNJREJ0TnlseTVFTld6NmtJQ3lOR2VLSkZFZUlqZTUydEdOZFUydFcxZVYyek1maHpCbw?oc=5</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>-0.34</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>-3.4</v>
+      </c>
+      <c r="H35" t="n">
+        <v>-5.100000000000001</v>
+      </c>
+      <c r="I35" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="J35" t="n">
+        <v>-1.7</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-02-08T17:15:11</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Aranceles de EE. UU. y puertos mexicanos: impacto, tensiones y respuestas del sector logístico - Tra</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Transporte.mx</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxPMjN3dzFjLW00S1BlRzlGUEZ0R2NKdkZlNVhnLXg4elg3QVU3NF80R3BhWEFuWWI0ZXdEaWFNaTl1WmUxX1hFYlpuUXZWV3F4Q210dVAwdk00NzRneWZmeWRkejRUNDhya0VaV1lYZkpRcEZ1cEZVeFh6RnV4SDJEQTdaNjBWS0RfXzNrbFF3NVFINFFDd21SZ19GMnlqLU1YaENzS1YtTGhlRjZDbzMxRnBJcw?oc=5</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>-0.34</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>-3.4</v>
+      </c>
+      <c r="H36" t="n">
+        <v>-5.100000000000001</v>
+      </c>
+      <c r="I36" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="J36" t="n">
+        <v>-1.7</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-02-08T11:19:14</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Aranceles a acero y aluminio afectarán precios de la construcción: CMIC Edomex - MSN</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>MSN</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi7gJBVV95cUxOR3h5N1RYZWNBb2pfQlR0dXczajZ1MXVyZmZ0U2VLbHk5OHd6bnkydUF0cWp0VHdjNEhZSUZyUm9xeUlYTXJRLWhheVNuSGxRa2RldEVWdUpWOEpHS0ZFWFd0R0VROHdyZDZTNEcybkh3NHFxbUVHY3QyTnBHcXZEZUJYZ1BxSWxmRWJQY1l3cFlza3lNendtZlNhUkF0OHFaWjdwekFvcnYyb3JZbDhpbTh2UEpGZDNwSGpDYzNBcGw4ZG04dlJEMUJCV2hJb09XZXllYXRFNnhsRm9mNDJGc3ZuNkdIQ1RLbmYtN3cwR04zWmh4em42aEt3dU1jaHFHbml2UHlFQUZQV0ZLWi13cDdqV2EzNGJxcDEyZTdoc0xWZVYwMll2b0dfMld6MlFxOVJESk9Xam81ejNNNWdsQXF1YW5mUGZSRkh3X3ZrSXhLTHJ1RnQxbzB0Y2xJdFlQZEZydHJDRWdGSEFpSnc?oc=5</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>-0.08000000000000002</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>-0.8000000000000002</v>
+      </c>
+      <c r="H37" t="n">
+        <v>-1.2</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0.4000000000000001</v>
+      </c>
+      <c r="J37" t="n">
+        <v>-0.4000000000000001</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-02-07T06:09:00</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Aranceles, despidos y silencio en la industria automotriz - El Heraldo de México</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>El Heraldo de México</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNa2l3SVJKUVZzVmNkcWVCOWJLQjBsMjRwWExMSlJyUkZDWTFiZ3lqelpxeUwtOVpKYmxNa2pYc3p5TE95ZG9oQ0ZCT1AxblNlck8yeWNvN0ZiYUk5bU84T0lVNW5RQVU5WmZqUDRmam8tb3BuV3QzejFkd05xcnJvVWxLYlhpN2wwUjBhQmdUUEFaUkt0bUs2VTZzekRqN0xfZmo2MnZPMzdPckNkU1R4ekEzRWrSAboBQVVfeXFMT2c5SUd2cE92ZnhQQnc2OF9GeWlLNmJKMUVKRFRnODRyNEdweTF2SzdGLVVGc0V5SWxkRWxOYjZXVjF4ZmdINU4zR3dqQU5ya2R5S092bjdhYXlWb3NOV2dwZHN1QnhlbFhRNHA4c1FkUkNkOE1fcnVPZzFNbC1lSVVXUGlNYl9Pc2hVRC00LWRndnVqVTlPN2NmVmZCVmNUS29PNERHWG41UGVOZkl1VEFvbUFrSVRMNEdn?oc=5</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>-0.34</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>-3.4</v>
+      </c>
+      <c r="H38" t="n">
+        <v>-5.100000000000001</v>
+      </c>
+      <c r="I38" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="J38" t="n">
+        <v>-1.7</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-02-07T04:33:00</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Acero, aluminio, minerales críticos y el financiamiento: los temas pendientes del acuerdo comercial </t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Infobae</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi5AFBVV95cUxPNWRtallwbGJmeTFLcXdUeHlXZzVNdzZ5dVFzSVRIU2lvTGtxX3dKVkVQX1Z4U1RDT0QxQm4zX3RJdTRiVzNUdzJ3Y1dOQms0bmdGMnF4aDVmSlZWT1ZweExCYTNrWE5pQ2wzejBDZi1wQnpHbkkzZzRDTjVSXzRtelJSekk0VkZCeU92X3BCdlV6TFRIMVZEeERuN2F6OUFrZVNQMndZMk9rNjRramtFSktQa3RHaEJkZ3VPeE0zTVZWUlhiUmR0Y0VMNXM2UjJjYm9MaUdTblpoeUhEanJaczF6b0_SAf8BQVVfeXFMTkNVXzJxVDVEakNYX3FSR2pHd1RmY0R1OU9XOVc5SGgwX3dqTExmNFpDQlNmRmJpMHYxWHNWc21LMG5mbFJ4dG50Wk9OR0pfeVRxdnJVOGNTbmpYN0sxUEpPRFU4Y3JaaUgxMVdKODVGa1Q0a0tOcllZOEVaYXFTUzlFNlpIX1VPdF9rMVpBYUg2TVBCSXotWGQ1Z0ozZzNUVnB2VEc3R0NoYlJzLW9xbnBfNWVuNXYxNnUwcnZTM2tJdFU1NjdKNWxRck5LNVVPUnBES1MtSDR2ZnF3Ylg2cU1rdkM4Qm4wSk5TR01fd2M4ekNybEh3ZjhURmJtcjg0?oc=5</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H39" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I39" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J39" t="n">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-02-06T17:41:00</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Acuerdo comercial: Pablo Quirno aseguró que EEUU se comprometió a revisar los aranceles al acero y a</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Ambito</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxQa0RLSjJObTlkcXJaQXozRjBHWUttWnQzM2ljRmJYclJtQzdPeTdBVzZqQWR0S0treWhIQURDM3ZJdEVzU1h5b0hhaUY3b0NCU3JSbVg2Y1lfeFFhU2RzOUt2aW5yX1ZyM0dYYjBJUFBZQmhoWjBrbTduUU5STUw0UzFyNFhHMFZwU0MzOU9feHFjNDhQTHJ4Tmk4ME5nUk92OU5OTE93S0ludXA4clNRdFMyMzdEazRfbU13d1hwMW1UaF9OUW9CRnBuYWh0VGd3WjNmb09sR3VoTWZQb2xjTW9B0gHnAUFVX3lxTE94aVhaTkJUQ0U5RDlCRHk5QVc3UWM0OWs2VjM5X3ZiNVVWT1JOekhITUpDWlc4YWRPS0dyS3FmTVFGZEQxdUJMMnA0RUwyUFAxRFE2T25WT3J5c0JwM1V3aVhtWE41QlQwZVNwWG1rUEJKY3Z0RXFsenUxTzdaXzVYMGZIV1BSSzhwaDZjMjVMRGRaS0lHbXp0anpUd2RIYzl2aGtwem82YlNFaUdQZXVCTzRTOEItMnhwY25CbmlYN2NFa1BaeEhoaHU4Rlh4eXAtOVRGY3VuUXhTVUw3aS03LTcyTnQxZw?oc=5</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>-0.34</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>-3.4</v>
+      </c>
+      <c r="H40" t="n">
+        <v>-5.100000000000001</v>
+      </c>
+      <c r="I40" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="J40" t="n">
+        <v>-1.7</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-02-06T17:30:00</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Carne, autopartes, acero, aluminio y otros puntos clave: cuáles son las definiciones que vendrán sob</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Infobae</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi9wFBVV95cUxQZXkweUpZSGZ4YzZ4VmJuaGtuMnFQWWpPSzZFc21pSjNJWXdldkpLRUxPQmdUOVF3MzJDXzVwck1TZGZCbE1CNVFtcDdUOHc3S3MzUGhkQTJFWTlsMjNBSEdJcnFfUFJKMm44MmRqT3RScnFUR3pmY3BPOC00Q0tzYXptc2p3bFkxQWhvdTM5LWN2ck01ekpkR2tUZ2QxSWlnSHVuekNxZDM2czA2Q2VhaTRUc3hnVXJXM3dVVF9UZjM2aGJDVjNFSXVTaUJkZEdEWkJPSHFYOGhqSnRHSlQzN0kyUUFDQ2h1cUdsZmJSUlp2bE1pemhZ0gGSAkFVX3lxTE9FT2k4S0dVdDJKNWxGSkZIb3VBYU5fMWY0b2VhSWM1QjF5T2RmSlJkM1hUSWhoYnVLWWhXeVN3TXpkeEZqY1BPWjNjSkFiRFR0SlpQQkFrVDd5VEhQUzk5bEYzMC1POHZ5ajhoaE1BZ3BiSlFlYWpMeGtWckcwNlh1eVJIbVNOLVYydEhORFZzUnFpcmN5eVE4cG9RTHFwSjlSS1djaE1qNVN3dFh3UEZiSlpudFlJTXMzV2lINUlIWmZiWXo1WlNUY2VJSllyMGxyRzgyUV9BeUdlcW43RUZQTUFvZWl1ZTdpNzV1YVA2aHNGN3FBWVg5TUk2UzRTcURZYmlxX0Y3UTRZUVZ6U0l6cnc?oc=5</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H41" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I41" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J41" t="n">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-02-06T17:26:58</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Diálogo y cooperación, fortaleza de relación entre México y Estados Unidos - El Diario de Sonora</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>El Diario de Sonora</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxQNTBILXVLc2NmOXNENms1NEowS2lfeVNRc1JYd1dUX0hLcVhSV183dnJzWWh5SW9MeF91Z25kMno3LW0wQ1ltVllZTWNJblFNbjFfQ3hrX0wtMHBaaXBzSkFrR3diTGdYX2pCeGV1ZzVYNEFkLXVoY216WFNwU0R1NDlSSk5WRnQzenlXb1owVlluUnlRZzhOVE5KQVlYZnFPWl9FUVdYZFcwR3NxTjNjOE1hWEZFWUU?oc=5</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H42" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I42" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J42" t="n">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-02-06T01:00:44</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Argentina firma acuerdo de comercio e inversión con EE.UU. - DW.com</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>DW.com</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxQV3NNdWcwQk1RMjFGMnkzUmVXbld4N29wX2N1d0ZBakdzNHBsWDV1NnVhY1ZOVHpEV0J2SzNQQURjdmRQaDhabkRXcTRxSjltcjQ3amJHQzZGSFBLVFRwRVoyLXFRQkpja2hZQS1XLV8wbmxoRlJ4UWxQRmMyTVpOcXNWOEhwYnpCdWc0NXFqUnJOOXhPS0owSkpB0gGaAUFVX3lxTE13NFZoWVpEYWdseWJOcUgtY1BoTkpqR0RIclNhaHpnUVp6dkdxdUZBcDFIM01CLTEydnhJVzd6MVpWUGNieGxOUXgyRm9tRGVWdnNuM3h5TnQ5YTlfWDJBRU5NR1NKQmlSWXJIQWZ6Q3hhQU9ZeWg0dWd1WEx1TG5mb1VzLTBGeDFwdmlzMVlBaVk5d0tlQS1YTGc?oc=5</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H43" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I43" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J43" t="n">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-02-06T00:26:00</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Reliquia del protomártir San Felipe de Jesús estrena lugar especial en la Catedral de la Ciudad de M</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>ACI Prensa</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxNeEUxUlVBbHMwclBWa0VOSlF4S2J1RVR1TGpxMEExeE1ZM3JxTnRaSkpaeUVlUzBVODdqYzVLeUtKZzhNcTNUMUZTaDJPN2ZtWXZFYUh4aWpXaDc1UnUyLXg5V3BvSGNUTW53QnFOLXQzWGpyeHJjYngxLVFBTHVyTFA2dGJ1OFhPN3Y5RGMtM1F3MXhfVXBtaXE3Zm5QalA1ZzNqZzNZTXVXVnNGczBxTURhbXdOT1A4bjdZNG1nTVZMZ0lG0gHKAUFVX3lxTE9KQy1UVFJNMVpwMFhrMGpXLXllRjladDlWT0hiZXRqRDdoZHIxNkRwSlRlNkcySEg5OXFpcjliTl9ZNHRWd1h3c2ZNQ1NOOHMwc0Jkb0FxMGZFMzNnOVFjWTlxQmF5T1RfbkxtX1VSdVpEV0RpLUtLb3BEZFdFOVBYaDZQODFHLVlrbVlkUWl5YW8tMjk4ZV8wTE8wdkFHTFVIYmFTb1o1UTZ0VHhKXzF6Rnlnd3JRUUl3MUU0MmVyQzZmdkpWUS1sQ3c?oc=5</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H44" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I44" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J44" t="n">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-02-06T00:00:00</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>El día después del acuerdo comercial con Estados Unidos: dólar estable y rebote la Bolsa porteña</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>La Nacion</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>https://www.lanacion.com.ar/economia/el-dia-despues-del-acuerdo-comercial-con-estados-unidos-dolar-estable-y-rebote-la-bolsa-portena-nid06022026/</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>-0.3200000000000001</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>-0.9600000000000002</v>
+      </c>
+      <c r="H45" t="n">
+        <v>-1.28</v>
+      </c>
+      <c r="I45" t="n">
+        <v>-0.6400000000000001</v>
+      </c>
+      <c r="J45" t="n">
+        <v>-1.6</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-02-05T19:01:53</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>El dinero que usas todos los días cambiará en 2026: así serán las nuevas monedas de 10 pesos en Méxi</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Xataka México</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQekdzejQ4OGZXTFhiYWtWVUFZeTk5eXJaNjhBUTZHX0hxSHZYM1hKVXFRX0MxUEJ1dXYzQWgzSndpVFYxTFpRNDBLbHdLWnVXeVY5X3l0Tk9ZTC01bjl6UFNaZDBIOHZrODR0dlpzd2lWUUNzWE1IdFhPOHFHSnhCOGtiVUtrLWF6RUhWRUEyemU5MzZuQVNzSGtBbi1wb3VUVXlKbWxXMTYyZDhLSmVqc2h0WDUwQdIBuwFBVV95cUxNRE5Gc29RQlBCZkExenE5MTREYWRjWlEzWndsYXNJb1dhRVE0WEdzbzByeWpubExzZGlmOUxVZUxrb0x1cDRZaklLX19meVhrVWh6RW0zUzFYeHpUYWNhWWx3XzJ3RzA5OXVlRWZKM0JUVTdtM1ZzYktCc3ByaXAyYmVnd3ZYckhiSlVkSURybWowVzloTmxIU2dzM3hpc3dLY0ZyQmZfVWV6MVJKOUcyajdiUXVwNVFYTVdz?oc=5</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H46" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I46" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J46" t="n">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-02-05T18:36:00</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Choque entre tráiler y auto particular deja dos muertos en la carretera México-Texcoco - La Jornada</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>La Jornada</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxQOVl2VjVIU3NIVWVCblRVdGFwclBXZExXeEJrcWYyc3EtbHpSR1NKQUNDYUFpNzdUSkV2Um5nVHFFNFVUR25WdDFHZno0YXYtVjJpeVB3LUdsVmNjLXhQTnB2UGUxZDZhSUhxMFNrS3ZVbFFtQVpScFhVb3ByT25aQnNhcjZTd1BRa1ppUVNtM3NaV2ZJQjZ6eEhubk96eHYtQ3ZSTDFoSU1ZV242QzJPZ1pRZy1rSFVhQWJtV21vUFRDVWduLUJwbWoxQ3FESHRFXzk0UUJB?oc=5</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="H47" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="I47" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="J47" t="n">
+        <v>1.04</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-02-05T17:07:00</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>México ante el injerencismo de Estados Unidos en Cuba - Cambio de Michoacán</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Cambio de Michoacán</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQS1AyRzFaejdCbXlISHQyR3NwbURiTXQzNmowWjY0ekFJb0RTaUZONWhrUW1MTWpZSU1FM3FPWFlVdzNZY3ZFZW9BUDdIYmVlVGY2X3kwUG9FZ19rLWFSTW9lRjlxZ3BiSzgzT0xZVGtZam1LNlZ0eWU3S19LSlZxTzRja0x5Z1VMcWo1QlJhUHgxZ2JVN2tMOGhXb3MxV2fSAacBQVVfeXFMT0hwTklVSXhVZFZRaEp6TXM1VHdGdll5a0xwWm84cEVDYmg5b0xEYWhOUkd5WWcxcVZFLXliS2VMUF94YW1nSXlSZ3hicHNpV3JiN3JSd3BzLXM0NjJJS3ptZHFhM2xZRzNRcTFucllqTVJWNThOTDRjdHRIdHhPNEkzQWM4cmlmNHNLbnpvZ1d5LWZUaURPeVNiRW9PRDU3ZUhRUmxydm8?oc=5</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H48" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I48" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J48" t="n">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-02-04T00:00:00</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Paolo Rocca sienta su postura sobre la licitación para el gasoducto de Vaca Muerta</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>La Nacion</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>https://www.lanacion.com.ar/politica/paolo-rocca-sienta-su-posicion-sobre-la-licitacion-de-tubos-para-el-gasoducto-de-vaca-muerta-nid04022026/</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>-0.04000000000000004</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>-0.1200000000000001</v>
+      </c>
+      <c r="H49" t="n">
+        <v>-0.4000000000000004</v>
+      </c>
+      <c r="I49" t="n">
+        <v>-0.08000000000000007</v>
+      </c>
+      <c r="J49" t="n">
+        <v>-0.08000000000000007</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-02-03T00:00:00</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Cuatro décadas de BASE</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>El Financiero</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>https://www.elfinanciero.com.mx/opinion/de-jefes/2026/02/03/cuatro-decadas-de-base/</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H50" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I50" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J50" t="n">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-02-02T00:00:00</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Mercados: caen bonos y acciones en el inicio de febrero, y rebota ligeramente el dólar</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>La Nacion</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>https://www.lanacion.com.ar/economia/dolar/mercados-caen-bonos-y-acciones-en-el-inicio-de-febrero-y-rebota-ligeramente-el-dolar-nid02022026/</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>-0.9239999999999999</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>negativo</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>-1.6632</v>
+      </c>
+      <c r="H51" t="n">
+        <v>-2.2176</v>
+      </c>
+      <c r="I51" t="n">
+        <v>-1.1088</v>
+      </c>
+      <c r="J51" t="n">
+        <v>-2.771999999999999</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-01-28T00:00:00</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Acereros y gobierno empujan blindaje de la región T-MEC rumbo a la revisión del tratado</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Milenio</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>https://www.milenio.com/negocios/acereros-gobierno-empujan-blindaje-revision-t-mec</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>-0.34</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G52" t="n">
+        <v>-3.4</v>
+      </c>
+      <c r="H52" t="n">
+        <v>-5.100000000000001</v>
+      </c>
+      <c r="I52" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="J52" t="n">
+        <v>-1.7</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-01-26T00:00:00</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Techint evalúa presentar un recurso antidumping contra la llegada de tubos de la India</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>La Nacion</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>https://www.lanacion.com.ar/economia/techint-evalua-presentar-un-recurso-antidumping-contra-la-llegada-de-tubos-de-la-india-nid26012026/</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>-0.6400000000000001</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G53" t="n">
+        <v>-6.400000000000001</v>
+      </c>
+      <c r="H53" t="n">
+        <v>-9.600000000000001</v>
+      </c>
+      <c r="I53" t="n">
+        <v>3.200000000000001</v>
+      </c>
+      <c r="J53" t="n">
+        <v>-3.200000000000001</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-01-23T00:00:00</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Tecnológica uruguaya Arkano sella alianza con brasileña Math Group y acelera expansión en el país no</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Diario EL PAIS Uruguay</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>https://www.elpais.com.uy/el-empresario/tecnologica-uruguaya-arkano-sella-alianza-con-brasilena-math-group-y-acelera-expansion-en-el-pais-norteno</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H54" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I54" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J54" t="n">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-01-15T00:00:00</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>ONU exige saber el paradero de activistas mexicanos desaparecidos hace 3 años</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Aristeguinoticias.com</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>https://aristeguinoticias.com/150126/mexico/onu-exige-saber-el-paradero-de-activistas-mexicanos-desaparecidos-hace-3-anos/</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G55" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H55" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I55" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J55" t="n">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-01-15T00:00:00</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Ternium adquirió Tubos Argentinos por US$24 millones y suma capacidad</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>La Nacion</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>https://www.lanacion.com.ar/economia/negocios/ternium-adquirio-tubos-argentinos-por-us24-millones-y-suma-capacidad-nid15012026/</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>0</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G56" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H56" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I56" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J56" t="n">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-01-14T00:00:00</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>CAP vende filial Tubos Argentinos a mayor grupo acerero de ese país</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Latercera.com</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>https://www.latercera.com/pulso/noticia/cap-vende-filial-tubos-argentinos-a-mayor-grupo-acerero-de-ese-pais/</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>0</v>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G57" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H57" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I57" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J57" t="n">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-01-14T00:00:00</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Grupo CAP vende acerera en Argentina en US$ 24,4 millones y sale del mercado trasandino</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Www.df.cl</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>https://www.df.cl/empresas/industria/grupo-cap-vende-acerera-en-argentina-y-sale-de-ese-mercado-para-enfocarse</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>0</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G58" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H58" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I58" t="n">
+        <v>-0</v>
+      </c>
+      <c r="J58" t="n">
+        <v>-0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Correcciones de RSS_Feed scraper
</commit_message>
<xml_diff>
--- a/Output/reporte_REAL.xlsx
+++ b/Output/reporte_REAL.xlsx
@@ -460,7 +460,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-02-12T09:51:45.540427</t>
+          <t>2026-02-12T10:10:22.868807</t>
         </is>
       </c>
     </row>
@@ -497,7 +497,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-1.165494736842105</v>
+        <v>-1.042687719298246</v>
       </c>
     </row>
     <row r="3">
@@ -507,7 +507,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-1.74899298245614</v>
+        <v>-1.55601052631579</v>
       </c>
     </row>
     <row r="4">
@@ -517,7 +517,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.5585298245614037</v>
+        <v>0.435722807017544</v>
       </c>
     </row>
     <row r="5">
@@ -527,7 +527,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.6666140350877193</v>
+        <v>-0.6139824561403509</v>
       </c>
     </row>
     <row r="6">
@@ -537,7 +537,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-1.394442105263158</v>
+        <v>-1.236547368421053</v>
       </c>
     </row>
   </sheetData>
@@ -1911,22 +1911,22 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-02-09T09:59:16</t>
+          <t>2026-02-09T14:01:02</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Tubos Reunidos registra unas pérdidas de 71,3 millones de euros por los aranceles estadounidenses al</t>
+          <t>El Chevrolet Onix 2026 baja de precio en México: más interesante que Aveo y ahora más barato - Motor</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>MSN</t>
+          <t>Motorpasión México</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-AFBVV95cUxQWGd2c3B3X3ZadU9tMnp3cWFWSmMySUdMT3ZKTUIxQXRnMmpfWFZfZ3MySlZaNUJJZHhhck01TFVQX3ZMelhNc1ZNQUFsYXVaODVkM0U5aUpzU0V1S01lcFgySDhzNkotUl83OFZVd2ZMd1dRcm9fclZXYVF0VVh0eUdkQ3hmQVhlaXkyQ25fNkxzRFB5d2tvWC13MEZhLVhYZjFjNlZZR3dhZmhQY1YyelQ0Q3JVRmxUUFpsRTRJR3RyS0pURXlaYUREM0ctajFwSkZxUHFITEY1VEwtbEJUbmxxNjVHM0pzNG5iQ1ctYW9RWkFRb29adg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE8zS0lrcFRsSkhCNmpodzZJU25nc3llWGx2d1J2ejNpMXVEQzBJUjZVX25STUg4WGxXNGRSZXVGTHR2WmJKUTREMUl2eEVzdnRFcmJLTUx1MFQ5X2FnOVBQV2JLQzBadGt4WDQ4blJfaUYzaTJicVN5aUpZdnQ2YknSAYQBQVVfeXFMTW53d3kyVG10MjNkVnkxUGJPaU42VzFvdzlpU1I3OEFuR0o4WHQzaVhkSU9HckJ3RFB4X0NZR2ZNR3k5VUFOd2wyQmxFS2txZUpYNTdyMzVtczhoWXdGbGo5UUlwMTFYNUJwR0ktR2J6YnM0bnh0bE56SndZeEJSVGpwc0JF?oc=5</t>
         </is>
       </c>
       <c r="E33" t="n">
@@ -1938,16 +1938,16 @@
         </is>
       </c>
       <c r="G33" t="n">
-        <v>-10</v>
+        <v>-3</v>
       </c>
       <c r="H33" t="n">
-        <v>-15</v>
+        <v>-4</v>
       </c>
       <c r="I33" t="n">
-        <v>5</v>
+        <v>-2</v>
       </c>
       <c r="J33" t="n">
-        <v>-5</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="34">
@@ -2336,12 +2336,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Argentina firma acuerdo de comercio e inversión con EE.UU. - DW.com</t>
+          <t>Argentina firma acuerdo de comercio e inversión con EE.UU. - dw.com</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>DW.com</t>
+          <t>dw.com</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">

</xml_diff>